<commit_message>
Fix ResourceAssignment FK and field set to match EC00630
Root cause analysis of fk_taskactv_task:
- Sample RA data had ActivityObjectId=68007 which is NOT in the
  5-sample activity set (67985-67989) — FK would always fail
- RA builder was missing 15+ fields present in EC00630:
  AtCompletionCost/Units, DrivingActivityDatesFlag, FinishDate,
  IsCostUnitsLinked, PlannedFinish/StartDate, PlannedLag,
  PlannedUnitsPerTime, Proficiency, RemainingDuration,
  RemainingFinish/StartDate, RemainingLag, RemainingUnitsPerTime,
  ResourceType, StartDate, UnitsPercentComplete, WBSObjectId
- ActivityObjectId was not first element (EC00630 puts it first)

Fixes:
- aurora_p6_converter.py: rebuild_resource_assignment_element rebuilt
  from scratch to match EC00630 field order and field set exactly
- create_template.py: RA sample filter now restricts to RAs whose
  ActivityObjectId is in the 5-sample activity set; added 8 new
  columns to ResourceAssignment sheet to cover new fields
</commit_message>
<xml_diff>
--- a/P6_Import_Template.xlsx
+++ b/P6_Import_Template.xlsx
@@ -8462,7 +8462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8470,16 +8470,23 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8500,62 +8507,97 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>ResourceType</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>RateType</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PlannedUnits</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PlannedCost</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PlannedUnitsPerTime</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PlannedStartDate</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PlannedFinishDate</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ActualUnits</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ActualCost</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RemainingUnits</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>RemainingCost</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>RemainingDuration</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>IsPrimaryResource</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Proficiency</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ObjectId</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>ActivityObjectId</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>ResourceObjectId</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>ProjectObjectId</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>WBSObjectId</t>
         </is>
       </c>
     </row>
@@ -8582,55 +8624,90 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Enum</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Enum</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>ObjectId</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>ObjectId</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>ObjectId</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>ObjectId</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>ObjectId</t>
         </is>
@@ -8642,192 +8719,97 @@
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>Price / Unit</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>81.000000</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>567.000000</t>
+          <t>172.800000</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>20736.000000</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>0.99884393</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>2015-02-18T13:48:00</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>2015-03-20T09:48:00</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
           <t>0.000000</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>0.000000</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>81.000000</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>567.000000</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>38990</t>
-        </is>
-      </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>68007</t>
+          <t>172.800000</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>2225</t>
+          <t>20736.000000</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
+          <t>173.00000011012731488491900832</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>3 - Skilled</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>38971</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>67989</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>2436</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
           <t>5232</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Price / Unit</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>81.000000</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>324.000000</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>0.000000</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>0.000000</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>81.000000</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>324.000000</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>38991</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>68007</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>2219</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>5232</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Price / Unit</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>81.000000</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>567.000000</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>0.000000</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>0.000000</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>81.000000</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>567.000000</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>38992</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>68007</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>2230</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>5232</t>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>17590</t>
         </is>
       </c>
     </row>

</xml_diff>